<commit_message>
fix(grimperium_mini): update default thread count and enhance progress tracking
- Increased the default thread count from 4 to 8 in the MiniConfig class to improve parallel processing capabilities.
- Modified the MiniProgressTracker to track the current molecule ID and display it in the progress table, enhancing user feedback during execution.
- Updated the progress table caption to show the number of completed and remaining tasks for better clarity.

These changes aim to optimize performance and improve the user experience during molecular processing.
</commit_message>
<xml_diff>
--- a/results/grimperium_mini_summary.xlsx
+++ b/results/grimperium_mini_summary.xlsx
@@ -160,8 +160,10 @@
           <t>CC(=O)O</t>
         </is>
       </c>
-      <c r="D3">
-        <v>0</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -193,14 +195,475 @@
           <t>dry_run</t>
         </is>
       </c>
-      <c r="K3">
-        <v>-432.2</v>
-      </c>
-      <c r="L3">
-        <v>0.0</v>
-      </c>
-      <c r="M3">
-        <v>0.0</v>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>-432.2</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cbt_001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Acetic acid</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CC(=O)O</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-431.09659904</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-426.94740992</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-427.59216432</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-432.2</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>18.3</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cbt_002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Propanoic acid</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-456.47038336</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>-445.09366896000006</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-446.53518248</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>-455.7</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>37.7</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cbt_003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Butyric acid</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-485.44491808</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>-468.01600584</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-468.51084752</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-475.8</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>73.5</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cbt_004</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pentanoic acid</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-511.6366744</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-488.50915416000004</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-488.38735792</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-491.3</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>119.8</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cbt_005</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Hexanoic acid</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-540.2830580000001</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-511.17333824</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-509.72303832</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-511.9</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>246.7</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cbt_006</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Heptanoic acid</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-568.96492192</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-533.87948784</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-531.13792184</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-536.2</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>431.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cbt_007</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Octanoic acid</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>345</v>
+      </c>
+      <c r="E10">
+        <v>-597.65519568</v>
+      </c>
+      <c r="F10">
+        <v>-556.59655768</v>
+      </c>
+      <c r="G10">
+        <v>-552.49581928</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K10">
+        <v>-556.0</v>
+      </c>
+      <c r="L10">
+        <v>811.8</v>
+      </c>
+      <c r="M10">
+        <v>13.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(grimperium_mini): enhance pipeline with completed molecule tracking and summary updates
- Introduced a new function to load completed molecule IDs from the summary Excel file, allowing the pipeline to skip already successful molecules.
- Updated the run_pipeline function to utilize the new loading mechanism, improving efficiency by avoiding redundant processing.
- Enhanced the MiniProgressTracker to count and display skipped molecules in the progress summary, providing better insights into the processing status.
- Adjusted the default timeout for the CREST step in the MiniConfig class to 82800 seconds for extended processing needs.

These changes aim to optimize the molecular processing workflow and improve user feedback during execution.
</commit_message>
<xml_diff>
--- a/results/grimperium_mini_summary.xlsx
+++ b/results/grimperium_mini_summary.xlsx
@@ -629,17 +629,25 @@
           <t>CCCCCCCC(=O)O</t>
         </is>
       </c>
-      <c r="D10">
-        <v>345</v>
-      </c>
-      <c r="E10">
-        <v>-597.65519568</v>
-      </c>
-      <c r="F10">
-        <v>-556.59655768</v>
-      </c>
-      <c r="G10">
-        <v>-552.49581928</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>345</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-597.65519568</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-556.59655768</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-552.49581928</t>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -656,14 +664,615 @@
           <t>success</t>
         </is>
       </c>
-      <c r="K10">
-        <v>-556.0</v>
-      </c>
-      <c r="L10">
-        <v>811.8</v>
-      </c>
-      <c r="M10">
-        <v>13.53</v>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-556.0</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>811.8</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>13.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cbt_001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Acetic acid</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CC(=O)O</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-431.09668272000005</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-426.94720072</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-427.59228984000003</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-432.2</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>13.4</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>0.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cbt_002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Propanoic acid</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-456.4704252</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-445.09366896000006</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-446.53518248</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-455.7</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>24.3</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>cbt_003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Butyric acid</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-485.44495992000003</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>-468.01596400000005</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-468.51076384000004</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-475.8</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>46.2</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>0.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cbt_004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pentanoic acid</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-511.63454056000006</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-488.50919600000003</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-488.38731608</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-491.3</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>75.7</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cbt_005</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hexanoic acid</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-540.2830998400001</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-511.17170648000007</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-509.73864464</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-511.9</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>167.1</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2.78</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cbt_006</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Heptanoic acid</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-568.96546584</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-533.87952968</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-531.13771264</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-536.2</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>295.7</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>4.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cbt_007</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Octanoic acid</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>356</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-597.65452624</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-556.59697608</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-552.4978276</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-556.0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>567.4</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>9.46</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cbt_008</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dodecanoic acid</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-702.8559762400001</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>-647.67487384</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-643.63835984</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>-642.0</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>4333.3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>72.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cbt_009</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tetradecanoic acid</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>not_attempted</t>
+        </is>
+      </c>
+      <c r="K19">
+        <v>-693.7</v>
+      </c>
+      <c r="L19">
+        <v>7200.8</v>
+      </c>
+      <c r="M19">
+        <v>120.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(grimperium_mini): add settings configuration and enhance user interaction
- Introduced a new settings menu in the MiniApp to allow users to modify timeout and maximum conformers interactively.
- Updated the MiniConfig class to set a default maximum conformers value and extended the timeout for the CREST step to one week.
- Enhanced the build_crest_command function to include the maximum conformers in the command if specified.
- Improved error handling in the run_crest function to provide clearer feedback on process outcomes, including timeout and partial results.

These changes aim to improve user experience by providing more control over configuration settings and enhancing the robustness of the processing pipeline.
</commit_message>
<xml_diff>
--- a/results/grimperium_mini_summary.xlsx
+++ b/results/grimperium_mini_summary.xlsx
@@ -1232,47 +1232,1655 @@
           <t>CCCCCCCCCCCCCC(=O)O</t>
         </is>
       </c>
-      <c r="D19">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>not_attempted</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-693.7</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>7200.8</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>120.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cbt_009</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Tetradecanoic acid</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>5442</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-759.84552896</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-693.31218856</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-687.44011192</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>-693.7</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>40280.3</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>671.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cbt_010</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hexadecanoic acid</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCCCCCC(=O)O</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>8260</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>-815.30214776</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-731.86866904</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-731.5685088800001</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>-737.1</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>48328.4</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>805.47</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cbt_011</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Methanol</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>-238.71289000000002</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-217.14470472</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>-204.75993920000002</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-200.94</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>19.8</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>0.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cbt_012</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ethanol</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CCO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>-268.83471936</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>-245.840334</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>-242.08063344</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>-234.95</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cbt_013</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Glycerol</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>C(C(CO)O)O</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>-690.3070305599999</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>-609.72164248</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>-611.15587584</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>-577.9</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>43.9</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cbt_014</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Propanol</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CCCO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-297.84205664</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>-268.20795616</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>-262.48813528</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>-254.6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>21.2</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cbt_015</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Butanol</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CCCCO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>-324.53585112</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>-289.35765776000005</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>-282.55167048</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>-275.1</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cbt_016</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Pentanol</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>CCCCCO</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>-353.15629392</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>-312.00912248</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>-303.80475872</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>-295.7</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>80.4</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cbt_017</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hexanol</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CCCCCCO</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-381.87644144000006</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>-334.76577296000005</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>-325.11705056000005</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>-316.2</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>151.3</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cbt_018</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Heptanol</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CCCCCCCO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>-410.56905824</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>-357.48443272000003</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>-346.39093328000007</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>-336.8</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>11284.1</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>188.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cbt_019</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Octanol</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CCCCCCCCO</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>954</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>-439.2764864</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>-380.22447272</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>-367.78606832</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>-357.3</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>515.7</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>8.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>cbt_020</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Methyl acetate</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>-403.84419872</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>-393.95769960000007</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>-405.05751688000004</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>-411.9</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>21.5</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>0.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>cbt_021</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Methyl propionate</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>-428.91221632</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>-411.79823376</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>-423.45686608</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>-427.5</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>45.8</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>0.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>cbt_022</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Methyl butyrate</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>CCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>-455.478608</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>-432.73580656</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>-444.7594092</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>-450.7</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>88.3</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>cbt_023</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Methyl pentanoate</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>-484.12176992</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>-455.36660232</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>-466.29073344000005</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>-471.1</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>159.4</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cbt_024</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Methyl hexanoate</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>-512.76639624</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>-478.03296208</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>-487.65327512</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>-492.2</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>303.2</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>5.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cbt_025</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Methyl heptanoate</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CCCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>-537.39555408</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>-495.83270224000006</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>-508.81398064</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>-515.5</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>557.7</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>9.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cbt_026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Methyl octanoate</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CCCCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>563</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>-562.93908328</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>-518.1351376800001</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>-531.3489628000001</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>-533.9</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>933.7</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>15.56</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cbt_027</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Methyl Dodecanoate</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>7664</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>-674.13825544</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>-613.51263936</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>-620.8584881600001</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>-617.9</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>9353.0</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>155.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>cbt_028</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Methyl Tetradecanoate</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>6802</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>-731.55917856</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>-658.96497944</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>-664.5516236</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>-656.9</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>41004.9</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>683.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>cbt_029</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Methyl Hexadecanoate</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCCCCCC(=O)OC</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>10743</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>-787.9695401600001</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>-696.30889488</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>-712.02052616</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>-665.6</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>47692.8</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>794.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>cbt_030</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Triacetin</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>CC(=O)OCC(COC(C)=O)OC(C)=O</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>-1139.52507752</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>-1093.54249912</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>-1184.9814760800002</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>-1245.0</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>1138.1</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>18.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>cbt_031</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tributyrin</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CCCC(=O)OCC(COC(=O)CCC)OC(=O)CCC</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>6040</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>-1298.6357776</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>-1227.0581231200001</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>-1322.6008928</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>-1388.9</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>10967.6</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>182.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>cbt_032</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Trilaurin</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CCCCCCCCCCCC(=O)OCC(COC(=O)CCCCCCCCCCC)OC(=O)CCCCCCCCCCC</t>
+        </is>
+      </c>
+      <c r="D43">
         <v>0</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>not_attempted</t>
         </is>
       </c>
-      <c r="K19">
-        <v>-693.7</v>
-      </c>
-      <c r="L19">
-        <v>7200.8</v>
-      </c>
-      <c r="M19">
-        <v>120.01</v>
+      <c r="K43">
+        <v>-1887.4899999999998</v>
+      </c>
+      <c r="L43">
+        <v>82808.8</v>
+      </c>
+      <c r="M43">
+        <v>1380.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>